<commit_message>
Auto commit 2026-07-13 23:47:19
</commit_message>
<xml_diff>
--- a/背景知识介绍/官方标准数据资料/股票样本.xlsx/股票样本.xlsx
+++ b/背景知识介绍/官方标准数据资料/股票样本.xlsx/股票样本.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026OPC大赛\自动化交易\股票样本.xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\2026OPC大赛\自动化交易\背景知识介绍\官方标准数据资料\股票样本.xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{663A9E12-11E9-47C7-A083-051F61150993}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8471AC67-11C5-498F-A9CD-E9E478B583B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>